<commit_message>
Chap 7, Ex 29, 30
</commit_message>
<xml_diff>
--- a/plan/Chapter7_ordered_schedule_actual_redo.xlsx
+++ b/plan/Chapter7_ordered_schedule_actual_redo.xlsx
@@ -1,42 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/plan/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="11_694932E1AE62AEE853A2737DE850B75DE210EBCF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{011A32EF-0172-45EB-B617-25EBEFE1C1DF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="19935" windowHeight="7935"/>
   </bookViews>
   <sheets>
     <sheet name="Master Schedule" sheetId="1" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
     <sheet name="Redo Rules" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="269">
   <si>
     <t>Order</t>
   </si>
@@ -659,6 +639,9 @@
     <t>7.37</t>
   </si>
   <si>
+    <t>Same as Ex 13</t>
+  </si>
+  <si>
     <t>Proceed gate: for every series problem, record the three series explicitly or say why a simpler criterion applies.</t>
   </si>
   <si>
@@ -840,20 +823,20 @@
   </si>
   <si>
     <t>Suggested Redo Date = Actual Start + offset. Actual End is automatically filled from Actual Redo Date.</t>
-  </si>
-  <si>
-    <t>Same as Ex 13</t>
-    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="5">
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -874,16 +857,157 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Carlito"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="Carlito"/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -908,8 +1032,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -917,52 +1227,339 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="49" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+  <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
+    <cellStyle name="输入" xfId="3" builtinId="20"/>
+    <cellStyle name="货币" xfId="4" builtinId="4"/>
+    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
+    <cellStyle name="差" xfId="7" builtinId="27"/>
+    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
+    <cellStyle name="超链接" xfId="10" builtinId="8"/>
+    <cellStyle name="百分比" xfId="11" builtinId="5"/>
+    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
+    <cellStyle name="注释" xfId="13" builtinId="10"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
+    <cellStyle name="标题" xfId="17" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
+    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
+    <cellStyle name="输出" xfId="24" builtinId="21"/>
+    <cellStyle name="计算" xfId="25" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
+    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
+    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
+    <cellStyle name="汇总" xfId="30" builtinId="25"/>
+    <cellStyle name="好" xfId="31" builtinId="26"/>
+    <cellStyle name="适中" xfId="32" builtinId="28"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
+    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
+    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
+    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
+    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <font>
-        <b/>
-      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFC6E0B4"/>
+          <bgColor rgb="FFFFE699"/>
         </patternFill>
       </fill>
     </dxf>
@@ -976,14 +1573,17 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFE699"/>
+          <bgColor rgb="FFC6E0B4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b val="1"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -993,54 +1593,43 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
   </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterScheduleTable" displayName="MasterScheduleTable" ref="A1:R64">
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Planned Date"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task Type"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Section(s)"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Task"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Exercise"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Related Result / Reason"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Prerequisite"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Proceed Gate"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Actual Start"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Actual End">
-      <calculatedColumnFormula>IF($P2&lt;&gt;"",$P2,"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="First-pass Status"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Key Blocker"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Suggested Redo Date (auto)">
-      <calculatedColumnFormula>IF(AND($C2="Exercise",$K2&lt;&gt;"",$M2&lt;&gt;""),$K2+VLOOKUP($M2,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Redo Result"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Proceed?"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Notes"/>
+    <tableColumn id="1" name="Order"/>
+    <tableColumn id="2" name="Planned Date"/>
+    <tableColumn id="3" name="Task Type"/>
+    <tableColumn id="4" name="Phase"/>
+    <tableColumn id="5" name="Section(s)"/>
+    <tableColumn id="6" name="Task"/>
+    <tableColumn id="7" name="Exercise"/>
+    <tableColumn id="8" name="Related Result / Reason"/>
+    <tableColumn id="9" name="Prerequisite"/>
+    <tableColumn id="10" name="Proceed Gate"/>
+    <tableColumn id="11" name="Actual Start"/>
+    <tableColumn id="12" name="Actual End"/>
+    <tableColumn id="13" name="First-pass Status"/>
+    <tableColumn id="14" name="Key Blocker"/>
+    <tableColumn id="15" name="Suggested Redo Date (auto)"/>
+    <tableColumn id="16" name="Redo Result"/>
+    <tableColumn id="17" name="Proceed?"/>
+    <tableColumn id="18" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RedoRulesTable" displayName="RedoRulesTable" ref="A1:D6">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="First-pass Status"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Meaning"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Recommended Action"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Redo Offset Days"/>
+    <tableColumn id="1" name="First-pass Status"/>
+    <tableColumn id="2" name="Meaning"/>
+    <tableColumn id="3" name="Recommended Action"/>
+    <tableColumn id="4" name="Redo Offset Days"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1189,14 +1778,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:S64"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1218,7 +1807,7 @@
     <col min="19" max="19" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="32.1" customHeight="1">
+    <row r="1" ht="32.1" customHeight="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1277,7 +1866,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="54">
+    <row r="2" ht="42.75" spans="1:19">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1318,7 +1907,7 @@
       <c r="R2" s="6"/>
       <c r="S2" s="4"/>
     </row>
-    <row r="3" spans="1:19" ht="54">
+    <row r="3" ht="42.75" spans="1:19">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1359,7 +1948,7 @@
       <c r="R3" s="6"/>
       <c r="S3" s="4"/>
     </row>
-    <row r="4" spans="1:19" ht="27">
+    <row r="4" ht="28.5" spans="1:19">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -1405,7 +1994,7 @@
       <c r="R4" s="6"/>
       <c r="S4" s="4"/>
     </row>
-    <row r="5" spans="1:19" ht="27">
+    <row r="5" ht="28.5" spans="1:19">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -1456,7 +2045,7 @@
       <c r="R5" s="6"/>
       <c r="S5" s="4"/>
     </row>
-    <row r="6" spans="1:19" ht="27">
+    <row r="6" ht="28.5" spans="1:19">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -1507,7 +2096,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="4"/>
     </row>
-    <row r="7" spans="1:19" ht="27">
+    <row r="7" ht="28.5" spans="1:19">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -1558,7 +2147,7 @@
       <c r="R7" s="6"/>
       <c r="S7" s="4"/>
     </row>
-    <row r="8" spans="1:19" ht="27">
+    <row r="8" ht="28.5" spans="1:19">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -1609,7 +2198,7 @@
       <c r="R8" s="6"/>
       <c r="S8" s="4"/>
     </row>
-    <row r="9" spans="1:19" ht="27">
+    <row r="9" ht="28.5" spans="1:19">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -1660,7 +2249,7 @@
       <c r="R9" s="6"/>
       <c r="S9" s="4"/>
     </row>
-    <row r="10" spans="1:19" ht="27">
+    <row r="10" spans="1:19">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -1711,7 +2300,7 @@
       <c r="R10" s="6"/>
       <c r="S10" s="4"/>
     </row>
-    <row r="11" spans="1:19" ht="27">
+    <row r="11" ht="28.5" spans="1:19">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -1762,7 +2351,7 @@
       <c r="R11" s="6"/>
       <c r="S11" s="4"/>
     </row>
-    <row r="12" spans="1:19" ht="54">
+    <row r="12" ht="57" spans="1:19">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -1811,7 +2400,7 @@
       <c r="R12" s="6"/>
       <c r="S12" s="4"/>
     </row>
-    <row r="13" spans="1:19" ht="40.5">
+    <row r="13" ht="42.75" spans="1:19">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -1853,7 +2442,7 @@
       <c r="R13" s="6"/>
       <c r="S13" s="4"/>
     </row>
-    <row r="14" spans="1:19" ht="40.5">
+    <row r="14" ht="28.5" spans="1:19">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -1904,7 +2493,7 @@
       <c r="R14" s="6"/>
       <c r="S14" s="4"/>
     </row>
-    <row r="15" spans="1:19" ht="27">
+    <row r="15" ht="28.5" spans="1:19">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -1955,7 +2544,7 @@
       <c r="R15" s="6"/>
       <c r="S15" s="4"/>
     </row>
-    <row r="16" spans="1:19" ht="27">
+    <row r="16" ht="28.5" spans="1:19">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -2006,7 +2595,7 @@
       <c r="R16" s="6"/>
       <c r="S16" s="4"/>
     </row>
-    <row r="17" spans="1:19" ht="40.5">
+    <row r="17" ht="28.5" spans="1:19">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2057,7 +2646,7 @@
       <c r="R17" s="6"/>
       <c r="S17" s="4"/>
     </row>
-    <row r="18" spans="1:19" ht="40.5">
+    <row r="18" ht="28.5" spans="1:19">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2110,7 +2699,7 @@
       <c r="R18" s="6"/>
       <c r="S18" s="4"/>
     </row>
-    <row r="19" spans="1:19" ht="27">
+    <row r="19" ht="28.5" spans="1:19">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2161,7 +2750,7 @@
       <c r="R19" s="6"/>
       <c r="S19" s="4"/>
     </row>
-    <row r="20" spans="1:19" ht="27">
+    <row r="20" ht="28.5" spans="1:19">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -2212,7 +2801,7 @@
       <c r="R20" s="6"/>
       <c r="S20" s="4"/>
     </row>
-    <row r="21" spans="1:19" ht="67.5">
+    <row r="21" ht="57" spans="1:19">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2258,7 +2847,7 @@
       <c r="R21" s="6"/>
       <c r="S21" s="4"/>
     </row>
-    <row r="22" spans="1:19" ht="40.5">
+    <row r="22" ht="42.75" spans="1:19">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -2300,7 +2889,7 @@
       <c r="R22" s="6"/>
       <c r="S22" s="4"/>
     </row>
-    <row r="23" spans="1:19" ht="40.5">
+    <row r="23" ht="42.75" spans="1:19">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2342,7 +2931,7 @@
       <c r="R23" s="6"/>
       <c r="S23" s="4"/>
     </row>
-    <row r="24" spans="1:19" ht="40.5">
+    <row r="24" ht="28.5" spans="1:19">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -2392,7 +2981,7 @@
       <c r="R24" s="6"/>
       <c r="S24" s="4"/>
     </row>
-    <row r="25" spans="1:19" ht="27">
+    <row r="25" ht="28.5" spans="1:19">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -2443,7 +3032,7 @@
       <c r="R25" s="6"/>
       <c r="S25" s="4"/>
     </row>
-    <row r="26" spans="1:19" ht="27">
+    <row r="26" ht="28.5" spans="1:19">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -2494,7 +3083,7 @@
       <c r="R26" s="6"/>
       <c r="S26" s="4"/>
     </row>
-    <row r="27" spans="1:19" ht="40.5">
+    <row r="27" ht="28.5" spans="1:19">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -2547,7 +3136,7 @@
       </c>
       <c r="S27" s="4"/>
     </row>
-    <row r="28" spans="1:19" ht="40.5">
+    <row r="28" ht="42.75" spans="1:19">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -2593,7 +3182,7 @@
       <c r="R28" s="6"/>
       <c r="S28" s="4"/>
     </row>
-    <row r="29" spans="1:19" ht="54">
+    <row r="29" ht="42.75" spans="1:19">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -2635,7 +3224,7 @@
       <c r="R29" s="6"/>
       <c r="S29" s="4"/>
     </row>
-    <row r="30" spans="1:19" ht="40.5">
+    <row r="30" ht="28.5" spans="1:19">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -2677,7 +3266,7 @@
       <c r="R30" s="6"/>
       <c r="S30" s="4"/>
     </row>
-    <row r="31" spans="1:19" ht="40.5">
+    <row r="31" ht="28.5" spans="1:19">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -2728,7 +3317,7 @@
       <c r="R31" s="6"/>
       <c r="S31" s="4"/>
     </row>
-    <row r="32" spans="1:19" ht="40.5">
+    <row r="32" ht="28.5" spans="1:19">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -2779,7 +3368,7 @@
       <c r="R32" s="6"/>
       <c r="S32" s="4"/>
     </row>
-    <row r="33" spans="1:19" ht="40.5">
+    <row r="33" ht="28.5" spans="1:19">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -2830,7 +3419,7 @@
       <c r="R33" s="6"/>
       <c r="S33" s="4"/>
     </row>
-    <row r="34" spans="1:19" ht="40.5">
+    <row r="34" ht="28.5" spans="1:19">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -2881,7 +3470,7 @@
       <c r="R34" s="6"/>
       <c r="S34" s="4"/>
     </row>
-    <row r="35" spans="1:19" ht="40.5">
+    <row r="35" ht="28.5" spans="1:19">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -2932,7 +3521,7 @@
       <c r="R35" s="6"/>
       <c r="S35" s="4"/>
     </row>
-    <row r="36" spans="1:19" ht="40.5">
+    <row r="36" ht="28.5" spans="1:19">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -2983,7 +3572,7 @@
       <c r="R36" s="6"/>
       <c r="S36" s="4"/>
     </row>
-    <row r="37" spans="1:19" ht="40.5">
+    <row r="37" ht="28.5" spans="1:19">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -3034,7 +3623,7 @@
       <c r="R37" s="6"/>
       <c r="S37" s="4"/>
     </row>
-    <row r="38" spans="1:19" ht="40.5">
+    <row r="38" ht="28.5" spans="1:19">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -3083,7 +3672,7 @@
       <c r="R38" s="6"/>
       <c r="S38" s="4"/>
     </row>
-    <row r="39" spans="1:19" ht="40.5">
+    <row r="39" ht="28.5" spans="1:19">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -3134,7 +3723,7 @@
       <c r="R39" s="6"/>
       <c r="S39" s="4"/>
     </row>
-    <row r="40" spans="1:19" ht="40.5">
+    <row r="40" ht="28.5" spans="1:19">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -3183,7 +3772,7 @@
       <c r="R40" s="6"/>
       <c r="S40" s="4"/>
     </row>
-    <row r="41" spans="1:19" ht="54">
+    <row r="41" ht="42.75" spans="1:19">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -3230,7 +3819,7 @@
       <c r="R41" s="6"/>
       <c r="S41" s="4"/>
     </row>
-    <row r="42" spans="1:19" ht="54">
+    <row r="42" ht="42.75" spans="1:19">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -3271,7 +3860,7 @@
       <c r="R42" s="6"/>
       <c r="S42" s="4"/>
     </row>
-    <row r="43" spans="1:19" ht="40.5">
+    <row r="43" ht="42.75" spans="1:19">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -3312,7 +3901,7 @@
       <c r="R43" s="6"/>
       <c r="S43" s="4"/>
     </row>
-    <row r="44" spans="1:19" ht="40.5">
+    <row r="44" ht="28.5" spans="1:19">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -3363,7 +3952,7 @@
       <c r="R44" s="6"/>
       <c r="S44" s="4"/>
     </row>
-    <row r="45" spans="1:19" ht="40.5">
+    <row r="45" ht="28.5" spans="1:19">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -3414,7 +4003,7 @@
       <c r="R45" s="6"/>
       <c r="S45" s="4"/>
     </row>
-    <row r="46" spans="1:19" ht="40.5">
+    <row r="46" ht="28.5" spans="1:19">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -3465,7 +4054,7 @@
       <c r="R46" s="6"/>
       <c r="S46" s="4"/>
     </row>
-    <row r="47" spans="1:19" ht="40.5">
+    <row r="47" ht="28.5" spans="1:19">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -3516,7 +4105,7 @@
       <c r="R47" s="6"/>
       <c r="S47" s="4"/>
     </row>
-    <row r="48" spans="1:19" ht="40.5">
+    <row r="48" ht="28.5" spans="1:19">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -3567,7 +4156,7 @@
       <c r="R48" s="6"/>
       <c r="S48" s="4"/>
     </row>
-    <row r="49" spans="1:19" ht="40.5">
+    <row r="49" ht="28.5" spans="1:19">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -3618,7 +4207,7 @@
       <c r="R49" s="6"/>
       <c r="S49" s="4"/>
     </row>
-    <row r="50" spans="1:19" ht="40.5">
+    <row r="50" ht="28.5" spans="1:19">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -3669,7 +4258,7 @@
       <c r="R50" s="6"/>
       <c r="S50" s="4"/>
     </row>
-    <row r="51" spans="1:19" ht="40.5">
+    <row r="51" ht="28.5" spans="1:19">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -3720,7 +4309,7 @@
       <c r="R51" s="6"/>
       <c r="S51" s="4"/>
     </row>
-    <row r="52" spans="1:19" ht="40.5">
+    <row r="52" ht="28.5" spans="1:19">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -3771,7 +4360,7 @@
       <c r="R52" s="6"/>
       <c r="S52" s="4"/>
     </row>
-    <row r="53" spans="1:19" ht="40.5">
+    <row r="53" ht="28.5" spans="1:19">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -3822,7 +4411,7 @@
       <c r="R53" s="6"/>
       <c r="S53" s="4"/>
     </row>
-    <row r="54" spans="1:19" ht="40.5">
+    <row r="54" ht="28.5" spans="1:19">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -3873,7 +4462,7 @@
       <c r="R54" s="6"/>
       <c r="S54" s="4"/>
     </row>
-    <row r="55" spans="1:19" ht="40.5">
+    <row r="55" ht="28.5" spans="1:19">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -3903,7 +4492,7 @@
       </c>
       <c r="J55" s="6"/>
       <c r="K55" s="7" t="s">
-        <v>268</v>
+        <v>207</v>
       </c>
       <c r="L55" s="7" t="str">
         <f t="shared" si="1"/>
@@ -3920,7 +4509,7 @@
       <c r="R55" s="6"/>
       <c r="S55" s="4"/>
     </row>
-    <row r="56" spans="1:19" ht="54">
+    <row r="56" ht="42.75" spans="1:19">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -3937,17 +4526,17 @@
         <v>174</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G56" s="6"/>
       <c r="H56" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K56" s="7">
         <v>46250</v>
@@ -3967,7 +4556,7 @@
       <c r="R56" s="6"/>
       <c r="S56" s="4"/>
     </row>
-    <row r="57" spans="1:19" ht="67.5">
+    <row r="57" ht="57" spans="1:19">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -3978,18 +4567,18 @@
         <v>19</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G57" s="6"/>
       <c r="H57" s="6"/>
       <c r="I57" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="J57" s="6"/>
       <c r="K57" s="7">
@@ -4010,7 +4599,7 @@
       <c r="R57" s="6"/>
       <c r="S57" s="4"/>
     </row>
-    <row r="58" spans="1:19" ht="40.5">
+    <row r="58" ht="28.5" spans="1:19">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -4021,22 +4610,22 @@
         <v>6</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J58" s="6"/>
       <c r="K58" s="7">
@@ -4061,7 +4650,7 @@
       <c r="R58" s="6"/>
       <c r="S58" s="4"/>
     </row>
-    <row r="59" spans="1:19" ht="27">
+    <row r="59" ht="28.5" spans="1:19">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -4072,22 +4661,22 @@
         <v>6</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F59" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="I59" s="6" t="s">
         <v>220</v>
-      </c>
-      <c r="G59" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="H59" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="I59" s="6" t="s">
-        <v>219</v>
       </c>
       <c r="J59" s="6"/>
       <c r="K59" s="7">
@@ -4110,7 +4699,7 @@
       <c r="R59" s="6"/>
       <c r="S59" s="4"/>
     </row>
-    <row r="60" spans="1:19" ht="27">
+    <row r="60" ht="28.5" spans="1:19">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -4121,41 +4710,45 @@
         <v>6</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J60" s="6"/>
-      <c r="K60" s="7"/>
+      <c r="K60" s="7">
+        <v>46266</v>
+      </c>
       <c r="L60" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M60" s="6"/>
+      <c r="M60" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N60" s="6"/>
-      <c r="O60" s="7" t="str">
+      <c r="O60" s="7">
         <f>IF(AND($C60="Exercise",$K60&lt;&gt;"",$M60&lt;&gt;""),$K60+VLOOKUP($M60,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46268</v>
       </c>
       <c r="P60" s="7"/>
       <c r="Q60" s="6"/>
       <c r="R60" s="6"/>
       <c r="S60" s="4"/>
     </row>
-    <row r="61" spans="1:19" ht="27">
+    <row r="61" ht="28.5" spans="1:19">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -4166,41 +4759,45 @@
         <v>6</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J61" s="6"/>
-      <c r="K61" s="7"/>
+      <c r="K61" s="7">
+        <v>46267</v>
+      </c>
       <c r="L61" s="7" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="M61" s="6"/>
+      <c r="M61" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="N61" s="6"/>
-      <c r="O61" s="7" t="str">
+      <c r="O61" s="7">
         <f>IF(AND($C61="Exercise",$K61&lt;&gt;"",$M61&lt;&gt;""),$K61+VLOOKUP($M61,'Redo Rules'!$A$2:$D$5,4,FALSE),"")</f>
-        <v/>
+        <v>46269</v>
       </c>
       <c r="P61" s="7"/>
       <c r="Q61" s="6"/>
       <c r="R61" s="6"/>
       <c r="S61" s="4"/>
     </row>
-    <row r="62" spans="1:19" ht="27">
+    <row r="62" ht="28.5" spans="1:19">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -4211,22 +4808,22 @@
         <v>6</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J62" s="6"/>
       <c r="K62" s="7"/>
@@ -4245,7 +4842,7 @@
       <c r="R62" s="6"/>
       <c r="S62" s="4"/>
     </row>
-    <row r="63" spans="1:19" ht="54">
+    <row r="63" ht="42.75" spans="1:19">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -4253,21 +4850,21 @@
         <v>46238</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="G63" s="6"/>
       <c r="H63" s="6"/>
       <c r="I63" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J63" s="6"/>
       <c r="K63" s="7"/>
@@ -4286,7 +4883,7 @@
       <c r="R63" s="6"/>
       <c r="S63" s="4"/>
     </row>
-    <row r="64" spans="1:19" ht="54">
+    <row r="64" ht="57" spans="1:19">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -4294,21 +4891,21 @@
         <v>46239</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G64" s="6"/>
       <c r="H64" s="6"/>
       <c r="I64" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J64" s="6"/>
       <c r="K64" s="7"/>
@@ -4328,35 +4925,35 @@
       <c r="S64" s="4"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="M2:M64">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$M2="Totally ignorance"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>$M2="Spark"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$M2="Skeleton"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>$M2="Crack it"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O64">
-    <cfRule type="expression" dxfId="0" priority="5">
+    <cfRule type="expression" dxfId="4" priority="5">
       <formula>AND($O2&lt;&gt;"",$O2&lt;=TODAY(),$P2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="M2:M64" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="M2:M64">
       <formula1>"Totally ignorance,Spark,Skeleton,Crack it"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="Q2:R64" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="Q2:R64">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -4364,109 +4961,110 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="27">
+    <row r="1" ht="30" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" ht="27">
+    <row r="2" ht="28.5" spans="1:2">
       <c r="A2" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" ht="15" spans="1:2">
       <c r="A4" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B4" s="4">
         <f>COUNTA('Master Schedule'!$A$2:$A$64)</f>
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" ht="15" spans="1:2">
       <c r="A5" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B5" s="4">
         <f>COUNTIF('Master Schedule'!$C$2:$C$64,"Read")</f>
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" ht="15" spans="1:2">
       <c r="A6" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Master Schedule'!$C$2:$C$64,"Exercise")</f>
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" ht="15" spans="1:2">
       <c r="A7" s="5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Master Schedule'!$C$2:$C$64,"Gate")</f>
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" ht="15" spans="1:2">
       <c r="A8" s="5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Master Schedule'!$C$2:$C$64,"Summary")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="27">
+    <row r="9" ht="15" spans="1:2">
       <c r="A9" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Master Schedule'!$P$2:$P$64,"&gt;0")</f>
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="27">
+    <row r="10" ht="15" spans="1:2">
       <c r="A10" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B10" s="4">
         <f ca="1">COUNTIFS('Master Schedule'!$O$2:$O$64,"&lt;="&amp;TODAY(),'Master Schedule'!$O$2:$O$64,"&gt;0",'Master Schedule'!$Q$2:$Q$64,"&lt;&gt;Y")</f>
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" ht="15" spans="1:2">
       <c r="A12" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B12" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Totally ignorance")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" ht="15" spans="1:2">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
@@ -4475,7 +5073,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" ht="15" spans="1:2">
       <c r="A14" s="5" t="s">
         <v>39</v>
       </c>
@@ -4484,45 +5082,46 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" ht="15" spans="1:2">
       <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B15" s="4">
         <f>COUNTIF('Master Schedule'!$M$2:$M$64,"Crack it")</f>
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
     </row>
-    <row r="17" spans="1:2" ht="27">
+    <row r="17" ht="15" spans="1:2">
       <c r="A17" s="5" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="18" ht="15" spans="1:2">
       <c r="A18" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
-  <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -4530,29 +5129,29 @@
     <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="27">
+    <row r="1" ht="15" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
@@ -4563,10 +5162,10 @@
         <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D3" s="2">
         <v>2</v>
@@ -4577,10 +5176,10 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D4" s="2">
         <v>2</v>
@@ -4591,29 +5190,29 @@
         <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C5" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D5" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
-  <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>